<commit_message>
Just installed proper modules, should take away errors for others looking at it
</commit_message>
<xml_diff>
--- a/Data/AutoData.xlsx
+++ b/Data/AutoData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Spring26\SP\SeniorProject\CustomerSide\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Spring26\SP\SeniorProject\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D06F087B-D00D-4821-8D23-893794E48C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE2B38C-D749-4ABC-861A-A61BE66D1BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="30912" windowHeight="16752" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ThisMonth" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -97,6 +97,21 @@
   </si>
   <si>
     <t>Oil Change</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>No-Show</t>
+  </si>
+  <si>
+    <t>Sundays</t>
   </si>
 </sst>
 </file>
@@ -104,7 +119,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -150,7 +165,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -158,16 +173,16 @@
   </cellStyles>
   <dxfs count="29">
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
@@ -258,9 +273,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}" name="tblThisMonth" displayName="tblThisMonth" ref="A1:L3" totalsRowShown="0">
-  <autoFilter ref="A1:L3" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}" name="tblThisMonth" displayName="tblThisMonth" ref="A1:P3" totalsRowShown="0">
+  <autoFilter ref="A1:P3" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{6EB0692A-0AAC-44A3-9108-53DA42DCD2C3}" name="ID"/>
     <tableColumn id="2" xr3:uid="{02A7FDC7-1096-42C4-9190-A3BF97B65769}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{0764CA94-AC50-439D-A876-EEBB70DA0A37}" name="LastName"/>
@@ -271,8 +286,12 @@
     <tableColumn id="8" xr3:uid="{E1B06AF3-DB87-49B5-977B-82B41142830A}" name="CarColor"/>
     <tableColumn id="9" xr3:uid="{B590DFEF-0EED-4ECA-ACDD-7AD95479C24B}" name="CarYear" dataDxfId="26"/>
     <tableColumn id="10" xr3:uid="{B6CC6C5B-4BAE-46CA-8D52-0541477E6A2E}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{DD09B0F3-3155-425D-A7AE-BF9703244AEA}" name="DateSubmitted" dataDxfId="24"/>
-    <tableColumn id="12" xr3:uid="{1A1C61E5-5022-4EA3-9A96-F17DF35EFB7D}" name="AppointmentDate" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{DD09B0F3-3155-425D-A7AE-BF9703244AEA}" name="DateSubmitted" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{1A1C61E5-5022-4EA3-9A96-F17DF35EFB7D}" name="AppointmentDate" dataDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{F554A1BA-4EEB-469B-A352-655DF64C225D}" name="Time"/>
+    <tableColumn id="14" xr3:uid="{B5A7BAF1-2A8C-4839-A07C-67F108A1AAEA}" name="Cancelled"/>
+    <tableColumn id="15" xr3:uid="{3AFF3342-A98E-44AF-92DE-EA2D7162E616}" name="Completed"/>
+    <tableColumn id="16" xr3:uid="{575FDD39-95CE-4FE2-99B8-F6CDAFB450EA}" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -367,10 +386,10 @@
   <autoFilter ref="A1:E2" xr:uid="{D20FF597-310B-4F82-AC65-E0671BDC8318}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{E7D5D0CB-F75B-42D9-AE23-FC2A5E4C7CA1}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{910F1BBD-775C-4650-92A5-080DBA60FB3C}" name="StartDate" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{460FB669-995B-490D-B7EE-88BDB2C87123}" name="EndDate" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{1467F11B-1470-442F-B4D7-B3F5B1174121}" name="StartTime" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{F9FC0C8A-286D-4A0A-9E88-8405B219285F}" name="EndTime" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{910F1BBD-775C-4650-92A5-080DBA60FB3C}" name="StartDate" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{460FB669-995B-490D-B7EE-88BDB2C87123}" name="EndDate" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{1467F11B-1470-442F-B4D7-B3F5B1174121}" name="StartTime" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{F9FC0C8A-286D-4A0A-9E88-8405B219285F}" name="EndTime" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -698,8 +717,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="14.796875" customWidth="1"/>
@@ -719,7 +738,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -756,8 +775,20 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -795,7 +826,7 @@
         <v>46111</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="E3" s="3"/>
     </row>
   </sheetData>
@@ -832,7 +863,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -900,7 +931,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -968,7 +999,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1036,7 +1067,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1084,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073C8F8E-56D4-4759-9B53-87C4A14D7ED7}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.59765625" style="1" customWidth="1"/>
@@ -1093,7 +1124,7 @@
     <col min="5" max="5" width="9.8984375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1108,6 +1139,9 @@
       </c>
       <c r="E1" s="5" t="s">
         <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Customer info pages
</commit_message>
<xml_diff>
--- a/Data/AutoData.xlsx
+++ b/Data/AutoData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Spring26\SP\SeniorProject\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE2B38C-D749-4ABC-861A-A61BE66D1BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5539428A-98FC-40D4-A838-693386B8EA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="30912" windowHeight="16752" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ThisMonth" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -173,6 +173,81 @@
   </cellStyles>
   <dxfs count="29">
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
@@ -183,81 +258,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -279,15 +279,15 @@
     <tableColumn id="1" xr3:uid="{6EB0692A-0AAC-44A3-9108-53DA42DCD2C3}" name="ID"/>
     <tableColumn id="2" xr3:uid="{02A7FDC7-1096-42C4-9190-A3BF97B65769}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{0764CA94-AC50-439D-A876-EEBB70DA0A37}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{BC99315C-BC6F-4A45-A174-5D1FDA770D11}" name="Phone" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{8882939D-A8BB-408D-B238-A0C8DB54F6AA}" name="Email" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="4" xr3:uid="{BC99315C-BC6F-4A45-A174-5D1FDA770D11}" name="Phone" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{8882939D-A8BB-408D-B238-A0C8DB54F6AA}" name="Email" dataDxfId="23" dataCellStyle="Hyperlink"/>
     <tableColumn id="6" xr3:uid="{ADFA1A41-CA10-45AE-B456-EE9384F51279}" name="CarMake"/>
     <tableColumn id="7" xr3:uid="{D4E52CE1-68CE-4073-85B2-3616A4774C1C}" name="CarType"/>
     <tableColumn id="8" xr3:uid="{E1B06AF3-DB87-49B5-977B-82B41142830A}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{B590DFEF-0EED-4ECA-ACDD-7AD95479C24B}" name="CarYear" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{B590DFEF-0EED-4ECA-ACDD-7AD95479C24B}" name="CarYear" dataDxfId="22"/>
     <tableColumn id="10" xr3:uid="{B6CC6C5B-4BAE-46CA-8D52-0541477E6A2E}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{DD09B0F3-3155-425D-A7AE-BF9703244AEA}" name="DateSubmitted" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{1A1C61E5-5022-4EA3-9A96-F17DF35EFB7D}" name="AppointmentDate" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{DD09B0F3-3155-425D-A7AE-BF9703244AEA}" name="DateSubmitted" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{1A1C61E5-5022-4EA3-9A96-F17DF35EFB7D}" name="AppointmentDate" dataDxfId="20"/>
     <tableColumn id="13" xr3:uid="{F554A1BA-4EEB-469B-A352-655DF64C225D}" name="Time"/>
     <tableColumn id="14" xr3:uid="{B5A7BAF1-2A8C-4839-A07C-67F108A1AAEA}" name="Cancelled"/>
     <tableColumn id="15" xr3:uid="{3AFF3342-A98E-44AF-92DE-EA2D7162E616}" name="Completed"/>
@@ -298,84 +298,100 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}" name="tblNextMonth" displayName="tblNextMonth" ref="A1:L3" totalsRowShown="0">
-  <autoFilter ref="A1:L3" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}" name="tblNextMonth" displayName="tblNextMonth" ref="A1:P3" totalsRowShown="0">
+  <autoFilter ref="A1:P3" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{D84B68CF-4B5B-4FC3-ACA5-78BA4EB3B153}" name="ID"/>
     <tableColumn id="2" xr3:uid="{0488BC54-7510-4EF0-A06E-BA4B6930738E}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{CCCF101C-39D1-4E90-8D3F-62CA8AE99F40}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{8033E655-17C3-49DB-B9D9-F1B885BF3E35}" name="Phone" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{67300D0D-55C9-447E-9642-9458E4FB616B}" name="Email" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{8033E655-17C3-49DB-B9D9-F1B885BF3E35}" name="Phone" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{67300D0D-55C9-447E-9642-9458E4FB616B}" name="Email" dataDxfId="18"/>
     <tableColumn id="6" xr3:uid="{FE9F8D95-21B8-4436-B8D3-C8192FDA7888}" name="CarMake"/>
     <tableColumn id="7" xr3:uid="{D2BFE8AE-FC24-4B39-A471-4B8AA1882E52}" name="CarType"/>
     <tableColumn id="8" xr3:uid="{B22386E0-1F40-4D42-BC91-72C7648510BB}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{FC2FB1B7-16B5-4140-8625-F0A367FEBD2E}" name="CarYear" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{FC2FB1B7-16B5-4140-8625-F0A367FEBD2E}" name="CarYear" dataDxfId="17"/>
     <tableColumn id="10" xr3:uid="{6B1AF41D-DF6D-4AA3-A97D-B7CEA6B24F31}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{B6EA152B-B5C0-4AD2-B887-77511B9BFC29}" name="DateSubmitted" dataDxfId="20"/>
-    <tableColumn id="12" xr3:uid="{DE8F1C74-D9BE-488B-AD38-DA7910279F85}" name="AppointmentDate" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{B6EA152B-B5C0-4AD2-B887-77511B9BFC29}" name="DateSubmitted" dataDxfId="16"/>
+    <tableColumn id="12" xr3:uid="{DE8F1C74-D9BE-488B-AD38-DA7910279F85}" name="AppointmentDate" dataDxfId="15"/>
+    <tableColumn id="13" xr3:uid="{3562A118-6270-45BE-879A-1C59D7A2A10F}" name="Time"/>
+    <tableColumn id="14" xr3:uid="{746E6FDF-BD13-4828-ACF8-503CB4DFD9D6}" name="Cancelled"/>
+    <tableColumn id="15" xr3:uid="{0495780A-E703-4426-9C98-972FF26BF398}" name="Completed"/>
+    <tableColumn id="16" xr3:uid="{0FB930C5-1074-4B2D-8DA2-203F6231F236}" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}" name="tblMonthPlus2" displayName="tblMonthPlus2" ref="A1:L2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:L2" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}" name="tblMonthPlus2" displayName="tblMonthPlus2" ref="A1:P2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:P2" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{87038649-E8D4-4A63-9878-65C93B079A6E}" name="ID"/>
     <tableColumn id="2" xr3:uid="{30805B92-2434-422F-B948-915D780436E9}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{1175A504-4352-4616-81E0-EB12B6423456}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{390A6DA6-396B-4CAA-8D32-8406D2F9F42C}" name="Phone" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{179B0347-88BD-414A-9713-71FE0A0005C2}" name="Email" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{390A6DA6-396B-4CAA-8D32-8406D2F9F42C}" name="Phone" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{179B0347-88BD-414A-9713-71FE0A0005C2}" name="Email" dataDxfId="13"/>
     <tableColumn id="6" xr3:uid="{C0178993-D99C-445D-B9B9-E5F87291EDB0}" name="CarMake"/>
     <tableColumn id="7" xr3:uid="{D0B6DA22-7EAE-4FAF-868A-4870792342DD}" name="CarType"/>
     <tableColumn id="8" xr3:uid="{328D59B5-EA12-4A66-B547-4B9ADC5BF30A}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{ECB0B604-7553-4A08-A93D-7F199B20C8D6}" name="CarYear" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{ECB0B604-7553-4A08-A93D-7F199B20C8D6}" name="CarYear" dataDxfId="12"/>
     <tableColumn id="10" xr3:uid="{74E4FB57-7034-4C09-A691-B14E8FDBD074}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{33D76C45-8B33-4704-9B56-6CAB90E1AF0D}" name="DateSubmitted" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{1EDAAD6E-2CEA-4318-9389-3E9052CF7C1B}" name="AppointmentDate" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{33D76C45-8B33-4704-9B56-6CAB90E1AF0D}" name="DateSubmitted" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{1EDAAD6E-2CEA-4318-9389-3E9052CF7C1B}" name="AppointmentDate" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{74F19710-E00B-4B42-918C-63856806E7C7}" name="Time"/>
+    <tableColumn id="14" xr3:uid="{B71D83C4-4D2A-4310-9341-36B293E55380}" name="Cancelled"/>
+    <tableColumn id="15" xr3:uid="{0ACA9286-49EA-42E2-897B-2CDE6E386E6E}" name="Completed"/>
+    <tableColumn id="16" xr3:uid="{046B7672-93AC-489F-94C8-AB3083DDD585}" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}" name="tblMonthPlus3" displayName="tblMonthPlus3" ref="A1:L2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:L2" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}" name="tblMonthPlus3" displayName="tblMonthPlus3" ref="A1:P2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:P2" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{2A1B5034-0D43-4BE9-876A-F5B66CE5731F}" name="ID"/>
     <tableColumn id="2" xr3:uid="{8CBFFCDC-DF88-4DE9-A774-3AB591C16C71}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{362889A2-23A1-4406-A907-0FD79FE8BA82}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{90F56E63-C1DC-4295-86CE-D8FD8E5DDCA9}" name="Phone" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{AB114323-DFD6-4C57-B086-01B4ECE44731}" name="Email" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{90F56E63-C1DC-4295-86CE-D8FD8E5DDCA9}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{AB114323-DFD6-4C57-B086-01B4ECE44731}" name="Email" dataDxfId="8"/>
     <tableColumn id="6" xr3:uid="{1C9B3C05-77A2-4F58-B69E-0F9DAAB568E3}" name="CarMake"/>
     <tableColumn id="7" xr3:uid="{481E62D6-1B7F-4FB3-A303-66D0ECBA8A42}" name="CarType"/>
     <tableColumn id="8" xr3:uid="{2C7632F7-746F-4414-B01F-6AFCA6DD4EF2}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{97E19127-2FCC-4491-B617-BB9AFB8C71C7}" name="CarYear" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{97E19127-2FCC-4491-B617-BB9AFB8C71C7}" name="CarYear" dataDxfId="7"/>
     <tableColumn id="10" xr3:uid="{D480589F-4C12-47AF-A73F-02B58AFA5E09}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{B94BCA66-2930-4B11-B84F-368D16A423C4}" name="DateSubmitted" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{0BA1FA0C-33E8-45E8-91E6-0E85EF8534F0}" name="AppointmentDate" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{B94BCA66-2930-4B11-B84F-368D16A423C4}" name="DateSubmitted" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{0BA1FA0C-33E8-45E8-91E6-0E85EF8534F0}" name="AppointmentDate" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{7AE2B856-B218-45E5-9746-E37A81ED35C9}" name="Time"/>
+    <tableColumn id="14" xr3:uid="{1737C278-868C-459C-AD38-CDF54C6D400C}" name="Cancelled"/>
+    <tableColumn id="15" xr3:uid="{50BF5CE3-71E4-4581-94B3-99503ED9C027}" name="Completed"/>
+    <tableColumn id="16" xr3:uid="{8D01ED94-F965-4D66-8D85-EE1A0A46F5BB}" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}" name="tblLastMonth" displayName="tblLastMonth" ref="A1:L2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:L2" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}" name="tblLastMonth" displayName="tblLastMonth" ref="A1:P2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:P2" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{616A9AEF-2FCE-4F2C-B128-942245014F14}" name="ID"/>
     <tableColumn id="2" xr3:uid="{2503B90C-D1C2-4823-9939-B471055C922F}" name="FirstName"/>
     <tableColumn id="3" xr3:uid="{6FA31BFD-1439-468E-840E-18E2DFF8F4F1}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{DE8FC8F7-5E8F-4D96-810A-AAE653A305E7}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{E280F3D9-F8C7-49D8-9D1D-D14A125811BB}" name="Email" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{DE8FC8F7-5E8F-4D96-810A-AAE653A305E7}" name="Phone" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{E280F3D9-F8C7-49D8-9D1D-D14A125811BB}" name="Email" dataDxfId="3"/>
     <tableColumn id="6" xr3:uid="{00D4B225-C17A-4EC3-80E4-C3D2B9C350D5}" name="CarMake"/>
     <tableColumn id="7" xr3:uid="{9BC19BFC-F711-4085-8E99-B3A8D02895AE}" name="CarType"/>
     <tableColumn id="8" xr3:uid="{792137EF-50AC-4A18-91DA-250B721B11AE}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{6BCCD0F3-83C5-48CB-9C79-E2315BDBA39C}" name="CarYear" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{6BCCD0F3-83C5-48CB-9C79-E2315BDBA39C}" name="CarYear" dataDxfId="2"/>
     <tableColumn id="10" xr3:uid="{F4510439-D588-4A08-9337-B16FB6BF9810}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{C9083DE3-4D49-4411-8C72-DDFA1D1EA35F}" name="DateSubmitted" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{48E5D8E0-D500-47A8-84AE-65F49B1D7AA8}" name="AppointmentDate" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{C9083DE3-4D49-4411-8C72-DDFA1D1EA35F}" name="DateSubmitted" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{48E5D8E0-D500-47A8-84AE-65F49B1D7AA8}" name="AppointmentDate" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{D18B8AB6-E1BB-4AB9-B323-C4D0C50A4994}" name="Time"/>
+    <tableColumn id="14" xr3:uid="{9435D878-C499-455C-981C-36F9C81C80AA}" name="Cancelled"/>
+    <tableColumn id="15" xr3:uid="{1C9DF852-5044-4F05-9241-C8A55138165A}" name="Completed"/>
+    <tableColumn id="16" xr3:uid="{AE94D5AE-C563-434B-AFBF-85573C259C86}" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -386,10 +402,10 @@
   <autoFilter ref="A1:E2" xr:uid="{D20FF597-310B-4F82-AC65-E0671BDC8318}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{E7D5D0CB-F75B-42D9-AE23-FC2A5E4C7CA1}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{910F1BBD-775C-4650-92A5-080DBA60FB3C}" name="StartDate" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{460FB669-995B-490D-B7EE-88BDB2C87123}" name="EndDate" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{1467F11B-1470-442F-B4D7-B3F5B1174121}" name="StartTime" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{F9FC0C8A-286D-4A0A-9E88-8405B219285F}" name="EndTime" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{910F1BBD-775C-4650-92A5-080DBA60FB3C}" name="StartDate" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{460FB669-995B-490D-B7EE-88BDB2C87123}" name="EndDate" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{1467F11B-1470-442F-B4D7-B3F5B1174121}" name="StartTime" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{F9FC0C8A-286D-4A0A-9E88-8405B219285F}" name="EndTime" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -843,7 +859,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A9A7B6-12D9-480B-ABCB-35F3583C2293}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
@@ -863,7 +879,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -899,6 +915,18 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -911,7 +939,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D4C191B-C703-424E-B5B4-B9CC241833E1}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
@@ -931,7 +959,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -967,6 +995,18 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -979,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A835F465-ED5C-471E-93B6-BA054D90EE5A}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
@@ -999,7 +1039,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1035,6 +1075,18 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1047,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E01ACCD-5698-4424-95D5-93F796623CB6}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
@@ -1067,7 +1119,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1103,6 +1155,18 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update row 2 via API
</commit_message>
<xml_diff>
--- a/Data/AutoData.xlsx
+++ b/Data/AutoData.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Spring26\SP\SeniorProject\Data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5539428A-98FC-40D4-A838-693386B8EA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776"/>
   </bookViews>
   <sheets>
-    <sheet name="ThisMonth" sheetId="1" r:id="rId1"/>
-    <sheet name="NextMonth" sheetId="2" r:id="rId2"/>
-    <sheet name="Month+2" sheetId="3" r:id="rId3"/>
-    <sheet name="Month+3" sheetId="4" r:id="rId4"/>
-    <sheet name="LastMonth" sheetId="5" r:id="rId5"/>
-    <sheet name="BlackoutRules" sheetId="6" r:id="rId6"/>
+    <sheet sheetId="1" name="ThisMonth" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="NextMonth" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Month+2" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Month+3" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="LastMonth" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="BlackoutRules" state="visible" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -63,6 +57,42 @@
     <t>AppointmentDate</t>
   </si>
   <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>No-Show</t>
+  </si>
+  <si>
+    <t>LocalTest</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>213-123-2331</t>
+  </si>
+  <si>
+    <t>jdoe@gmail.com</t>
+  </si>
+  <si>
+    <t>Toyota</t>
+  </si>
+  <si>
+    <t>Sedan</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Oil Change</t>
+  </si>
+  <si>
     <t>StartDate</t>
   </si>
   <si>
@@ -75,67 +105,38 @@
     <t>EndTime</t>
   </si>
   <si>
-    <t>213-123-2331</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>jdoe@gmail.com</t>
-  </si>
-  <si>
-    <t>Toyota</t>
-  </si>
-  <si>
-    <t>Sedan</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>Oil Change</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Cancelled</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>No-Show</t>
-  </si>
-  <si>
     <t>Sundays</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss AM/PM"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="12"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -155,112 +156,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-  </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -273,139 +184,230 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}" name="tblThisMonth" displayName="tblThisMonth" ref="A1:P3" totalsRowShown="0">
-  <autoFilter ref="A1:P3" xr:uid="{1CADB0E1-0277-4C20-B65A-62DC77B8AD95}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="tblThisMonth" displayName="tblThisMonth" ref="A1:P3" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P3">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{6EB0692A-0AAC-44A3-9108-53DA42DCD2C3}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{02A7FDC7-1096-42C4-9190-A3BF97B65769}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{0764CA94-AC50-439D-A876-EEBB70DA0A37}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{BC99315C-BC6F-4A45-A174-5D1FDA770D11}" name="Phone" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{8882939D-A8BB-408D-B238-A0C8DB54F6AA}" name="Email" dataDxfId="23" dataCellStyle="Hyperlink"/>
-    <tableColumn id="6" xr3:uid="{ADFA1A41-CA10-45AE-B456-EE9384F51279}" name="CarMake"/>
-    <tableColumn id="7" xr3:uid="{D4E52CE1-68CE-4073-85B2-3616A4774C1C}" name="CarType"/>
-    <tableColumn id="8" xr3:uid="{E1B06AF3-DB87-49B5-977B-82B41142830A}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{B590DFEF-0EED-4ECA-ACDD-7AD95479C24B}" name="CarYear" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{B6CC6C5B-4BAE-46CA-8D52-0541477E6A2E}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{DD09B0F3-3155-425D-A7AE-BF9703244AEA}" name="DateSubmitted" dataDxfId="21"/>
-    <tableColumn id="12" xr3:uid="{1A1C61E5-5022-4EA3-9A96-F17DF35EFB7D}" name="AppointmentDate" dataDxfId="20"/>
-    <tableColumn id="13" xr3:uid="{F554A1BA-4EEB-469B-A352-655DF64C225D}" name="Time"/>
-    <tableColumn id="14" xr3:uid="{B5A7BAF1-2A8C-4839-A07C-67F108A1AAEA}" name="Cancelled"/>
-    <tableColumn id="15" xr3:uid="{3AFF3342-A98E-44AF-92DE-EA2D7162E616}" name="Completed"/>
-    <tableColumn id="16" xr3:uid="{575FDD39-95CE-4FE2-99B8-F6CDAFB450EA}" name="No-Show"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Phone"/>
+    <tableColumn id="5" name="Email"/>
+    <tableColumn id="6" name="CarMake"/>
+    <tableColumn id="7" name="CarType"/>
+    <tableColumn id="8" name="CarColor"/>
+    <tableColumn id="9" name="CarYear"/>
+    <tableColumn id="10" name="ServiceType"/>
+    <tableColumn id="11" name="DateSubmitted"/>
+    <tableColumn id="12" name="AppointmentDate"/>
+    <tableColumn id="13" name="Time"/>
+    <tableColumn id="14" name="Cancelled"/>
+    <tableColumn id="15" name="Completed"/>
+    <tableColumn id="16" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}" name="tblNextMonth" displayName="tblNextMonth" ref="A1:P3" totalsRowShown="0">
-  <autoFilter ref="A1:P3" xr:uid="{025173BA-4ED8-4AAF-BF9A-05FE2A31C2F7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="tblNextMonth" displayName="tblNextMonth" ref="A1:P3" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P3">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{D84B68CF-4B5B-4FC3-ACA5-78BA4EB3B153}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{0488BC54-7510-4EF0-A06E-BA4B6930738E}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{CCCF101C-39D1-4E90-8D3F-62CA8AE99F40}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{8033E655-17C3-49DB-B9D9-F1B885BF3E35}" name="Phone" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{67300D0D-55C9-447E-9642-9458E4FB616B}" name="Email" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{FE9F8D95-21B8-4436-B8D3-C8192FDA7888}" name="CarMake"/>
-    <tableColumn id="7" xr3:uid="{D2BFE8AE-FC24-4B39-A471-4B8AA1882E52}" name="CarType"/>
-    <tableColumn id="8" xr3:uid="{B22386E0-1F40-4D42-BC91-72C7648510BB}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{FC2FB1B7-16B5-4140-8625-F0A367FEBD2E}" name="CarYear" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{6B1AF41D-DF6D-4AA3-A97D-B7CEA6B24F31}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{B6EA152B-B5C0-4AD2-B887-77511B9BFC29}" name="DateSubmitted" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{DE8F1C74-D9BE-488B-AD38-DA7910279F85}" name="AppointmentDate" dataDxfId="15"/>
-    <tableColumn id="13" xr3:uid="{3562A118-6270-45BE-879A-1C59D7A2A10F}" name="Time"/>
-    <tableColumn id="14" xr3:uid="{746E6FDF-BD13-4828-ACF8-503CB4DFD9D6}" name="Cancelled"/>
-    <tableColumn id="15" xr3:uid="{0495780A-E703-4426-9C98-972FF26BF398}" name="Completed"/>
-    <tableColumn id="16" xr3:uid="{0FB930C5-1074-4B2D-8DA2-203F6231F236}" name="No-Show"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Phone"/>
+    <tableColumn id="5" name="Email"/>
+    <tableColumn id="6" name="CarMake"/>
+    <tableColumn id="7" name="CarType"/>
+    <tableColumn id="8" name="CarColor"/>
+    <tableColumn id="9" name="CarYear"/>
+    <tableColumn id="10" name="ServiceType"/>
+    <tableColumn id="11" name="DateSubmitted"/>
+    <tableColumn id="12" name="AppointmentDate"/>
+    <tableColumn id="13" name="Time"/>
+    <tableColumn id="14" name="Cancelled"/>
+    <tableColumn id="15" name="Completed"/>
+    <tableColumn id="16" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}" name="tblMonthPlus2" displayName="tblMonthPlus2" ref="A1:P2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:P2" xr:uid="{59488172-1FFE-4304-B91F-AE627D0DF25C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" name="tblMonthPlus2" displayName="tblMonthPlus2" ref="A1:P2" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P2">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{87038649-E8D4-4A63-9878-65C93B079A6E}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{30805B92-2434-422F-B948-915D780436E9}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{1175A504-4352-4616-81E0-EB12B6423456}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{390A6DA6-396B-4CAA-8D32-8406D2F9F42C}" name="Phone" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{179B0347-88BD-414A-9713-71FE0A0005C2}" name="Email" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{C0178993-D99C-445D-B9B9-E5F87291EDB0}" name="CarMake"/>
-    <tableColumn id="7" xr3:uid="{D0B6DA22-7EAE-4FAF-868A-4870792342DD}" name="CarType"/>
-    <tableColumn id="8" xr3:uid="{328D59B5-EA12-4A66-B547-4B9ADC5BF30A}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{ECB0B604-7553-4A08-A93D-7F199B20C8D6}" name="CarYear" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{74E4FB57-7034-4C09-A691-B14E8FDBD074}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{33D76C45-8B33-4704-9B56-6CAB90E1AF0D}" name="DateSubmitted" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{1EDAAD6E-2CEA-4318-9389-3E9052CF7C1B}" name="AppointmentDate" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{74F19710-E00B-4B42-918C-63856806E7C7}" name="Time"/>
-    <tableColumn id="14" xr3:uid="{B71D83C4-4D2A-4310-9341-36B293E55380}" name="Cancelled"/>
-    <tableColumn id="15" xr3:uid="{0ACA9286-49EA-42E2-897B-2CDE6E386E6E}" name="Completed"/>
-    <tableColumn id="16" xr3:uid="{046B7672-93AC-489F-94C8-AB3083DDD585}" name="No-Show"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Phone"/>
+    <tableColumn id="5" name="Email"/>
+    <tableColumn id="6" name="CarMake"/>
+    <tableColumn id="7" name="CarType"/>
+    <tableColumn id="8" name="CarColor"/>
+    <tableColumn id="9" name="CarYear"/>
+    <tableColumn id="10" name="ServiceType"/>
+    <tableColumn id="11" name="DateSubmitted"/>
+    <tableColumn id="12" name="AppointmentDate"/>
+    <tableColumn id="13" name="Time"/>
+    <tableColumn id="14" name="Cancelled"/>
+    <tableColumn id="15" name="Completed"/>
+    <tableColumn id="16" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}" name="tblMonthPlus3" displayName="tblMonthPlus3" ref="A1:P2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:P2" xr:uid="{F4901B33-E49B-426F-81EA-4C138E0F80D0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" name="tblMonthPlus3" displayName="tblMonthPlus3" ref="A1:P2" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P2">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{2A1B5034-0D43-4BE9-876A-F5B66CE5731F}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{8CBFFCDC-DF88-4DE9-A774-3AB591C16C71}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{362889A2-23A1-4406-A907-0FD79FE8BA82}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{90F56E63-C1DC-4295-86CE-D8FD8E5DDCA9}" name="Phone" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{AB114323-DFD6-4C57-B086-01B4ECE44731}" name="Email" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{1C9B3C05-77A2-4F58-B69E-0F9DAAB568E3}" name="CarMake"/>
-    <tableColumn id="7" xr3:uid="{481E62D6-1B7F-4FB3-A303-66D0ECBA8A42}" name="CarType"/>
-    <tableColumn id="8" xr3:uid="{2C7632F7-746F-4414-B01F-6AFCA6DD4EF2}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{97E19127-2FCC-4491-B617-BB9AFB8C71C7}" name="CarYear" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{D480589F-4C12-47AF-A73F-02B58AFA5E09}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{B94BCA66-2930-4B11-B84F-368D16A423C4}" name="DateSubmitted" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{0BA1FA0C-33E8-45E8-91E6-0E85EF8534F0}" name="AppointmentDate" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{7AE2B856-B218-45E5-9746-E37A81ED35C9}" name="Time"/>
-    <tableColumn id="14" xr3:uid="{1737C278-868C-459C-AD38-CDF54C6D400C}" name="Cancelled"/>
-    <tableColumn id="15" xr3:uid="{50BF5CE3-71E4-4581-94B3-99503ED9C027}" name="Completed"/>
-    <tableColumn id="16" xr3:uid="{8D01ED94-F965-4D66-8D85-EE1A0A46F5BB}" name="No-Show"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Phone"/>
+    <tableColumn id="5" name="Email"/>
+    <tableColumn id="6" name="CarMake"/>
+    <tableColumn id="7" name="CarType"/>
+    <tableColumn id="8" name="CarColor"/>
+    <tableColumn id="9" name="CarYear"/>
+    <tableColumn id="10" name="ServiceType"/>
+    <tableColumn id="11" name="DateSubmitted"/>
+    <tableColumn id="12" name="AppointmentDate"/>
+    <tableColumn id="13" name="Time"/>
+    <tableColumn id="14" name="Cancelled"/>
+    <tableColumn id="15" name="Completed"/>
+    <tableColumn id="16" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}" name="tblLastMonth" displayName="tblLastMonth" ref="A1:P2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:P2" xr:uid="{A546873F-E386-42EC-8D1B-F659A4DD568F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" name="tblLastMonth" displayName="tblLastMonth" ref="A1:P2" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:P2">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{616A9AEF-2FCE-4F2C-B128-942245014F14}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{2503B90C-D1C2-4823-9939-B471055C922F}" name="FirstName"/>
-    <tableColumn id="3" xr3:uid="{6FA31BFD-1439-468E-840E-18E2DFF8F4F1}" name="LastName"/>
-    <tableColumn id="4" xr3:uid="{DE8FC8F7-5E8F-4D96-810A-AAE653A305E7}" name="Phone" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{E280F3D9-F8C7-49D8-9D1D-D14A125811BB}" name="Email" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{00D4B225-C17A-4EC3-80E4-C3D2B9C350D5}" name="CarMake"/>
-    <tableColumn id="7" xr3:uid="{9BC19BFC-F711-4085-8E99-B3A8D02895AE}" name="CarType"/>
-    <tableColumn id="8" xr3:uid="{792137EF-50AC-4A18-91DA-250B721B11AE}" name="CarColor"/>
-    <tableColumn id="9" xr3:uid="{6BCCD0F3-83C5-48CB-9C79-E2315BDBA39C}" name="CarYear" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{F4510439-D588-4A08-9337-B16FB6BF9810}" name="ServiceType"/>
-    <tableColumn id="11" xr3:uid="{C9083DE3-4D49-4411-8C72-DDFA1D1EA35F}" name="DateSubmitted" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{48E5D8E0-D500-47A8-84AE-65F49B1D7AA8}" name="AppointmentDate" dataDxfId="0"/>
-    <tableColumn id="13" xr3:uid="{D18B8AB6-E1BB-4AB9-B323-C4D0C50A4994}" name="Time"/>
-    <tableColumn id="14" xr3:uid="{9435D878-C499-455C-981C-36F9C81C80AA}" name="Cancelled"/>
-    <tableColumn id="15" xr3:uid="{1C9DF852-5044-4F05-9241-C8A55138165A}" name="Completed"/>
-    <tableColumn id="16" xr3:uid="{AE94D5AE-C563-434B-AFBF-85573C259C86}" name="No-Show"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="FirstName"/>
+    <tableColumn id="3" name="LastName"/>
+    <tableColumn id="4" name="Phone"/>
+    <tableColumn id="5" name="Email"/>
+    <tableColumn id="6" name="CarMake"/>
+    <tableColumn id="7" name="CarType"/>
+    <tableColumn id="8" name="CarColor"/>
+    <tableColumn id="9" name="CarYear"/>
+    <tableColumn id="10" name="ServiceType"/>
+    <tableColumn id="11" name="DateSubmitted"/>
+    <tableColumn id="12" name="AppointmentDate"/>
+    <tableColumn id="13" name="Time"/>
+    <tableColumn id="14" name="Cancelled"/>
+    <tableColumn id="15" name="Completed"/>
+    <tableColumn id="16" name="No-Show"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D20FF597-310B-4F82-AC65-E0671BDC8318}" name="tblBlackoutRules" displayName="tblBlackoutRules" ref="A1:E2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:E2" xr:uid="{D20FF597-310B-4F82-AC65-E0671BDC8318}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" name="tblBlackoutRules" displayName="tblBlackoutRules" ref="A1:E2" totalsRowShown="1" headerRowCount="0">
+  <autoFilter ref="A1:E2">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E7D5D0CB-F75B-42D9-AE23-FC2A5E4C7CA1}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{910F1BBD-775C-4650-92A5-080DBA60FB3C}" name="StartDate" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{460FB669-995B-490D-B7EE-88BDB2C87123}" name="EndDate" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{1467F11B-1470-442F-B4D7-B3F5B1174121}" name="StartTime" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{F9FC0C8A-286D-4A0A-9E88-8405B219285F}" name="EndTime" dataDxfId="25"/>
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="StartDate"/>
+    <tableColumn id="3" name="EndDate"/>
+    <tableColumn id="4" name="StartTime"/>
+    <tableColumn id="5" name="EndTime"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -732,21 +734,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="14.796875" customWidth="1"/>
-    <col min="4" max="4" width="15.09765625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.09765625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.5" customWidth="1"/>
     <col min="7" max="7" width="12.5" customWidth="1"/>
     <col min="8" max="8" width="12.3984375" customWidth="1"/>
-    <col min="9" max="9" width="9.796875" style="4" customWidth="1"/>
+    <col min="9" max="9" width="9.796875" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="21" width="10.09765625" customWidth="1"/>
     <col min="22" max="111" width="11.09765625" customWidth="1"/>
     <col min="112" max="1011" width="12.09765625" customWidth="1"/>
@@ -754,7 +756,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -764,10 +766,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -779,45 +781,45 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F2" t="s">
@@ -829,49 +831,49 @@
       <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="2">
         <v>2012</v>
       </c>
       <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="3">
         <v>46106</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="3">
         <v>46111</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="E3" s="3"/>
+    <row r="3" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E3" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{97E9D3E5-8A7D-4DD9-9584-E3619EEDCC2D}"/>
+    <hyperlink ref="E2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A9A7B6-12D9-480B-ABCB-35F3583C2293}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="10.796875" customWidth="1"/>
-    <col min="4" max="5" width="8.796875" style="2"/>
+    <col min="4" max="5" width="8.796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.09765625" customWidth="1"/>
     <col min="7" max="7" width="9.3984375" customWidth="1"/>
     <col min="8" max="8" width="9.8984375" customWidth="1"/>
-    <col min="9" max="9" width="9.09765625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="9.09765625" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="21" width="10.09765625" customWidth="1"/>
     <col min="22" max="111" width="11.09765625" customWidth="1"/>
     <col min="112" max="1011" width="12.09765625" customWidth="1"/>
@@ -879,7 +881,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -889,10 +891,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -904,29 +906,29 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -938,20 +940,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D4C191B-C703-424E-B5B4-B9CC241833E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="10.796875" customWidth="1"/>
-    <col min="4" max="5" width="8.796875" style="2"/>
+    <col min="4" max="5" width="8.796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.09765625" customWidth="1"/>
     <col min="7" max="7" width="9.3984375" customWidth="1"/>
     <col min="8" max="8" width="9.8984375" customWidth="1"/>
-    <col min="9" max="9" width="9.09765625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="9.09765625" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="21" width="10.09765625" customWidth="1"/>
     <col min="22" max="111" width="11.09765625" customWidth="1"/>
     <col min="112" max="1011" width="12.09765625" customWidth="1"/>
@@ -959,7 +961,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -969,10 +971,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -984,29 +986,29 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1018,20 +1020,20 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A835F465-ED5C-471E-93B6-BA054D90EE5A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="10.796875" customWidth="1"/>
-    <col min="4" max="5" width="8.796875" style="2"/>
+    <col min="4" max="5" width="8.796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.09765625" customWidth="1"/>
     <col min="7" max="7" width="9.3984375" customWidth="1"/>
     <col min="8" max="8" width="9.8984375" customWidth="1"/>
-    <col min="9" max="9" width="9.09765625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="9.09765625" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="21" width="10.09765625" customWidth="1"/>
     <col min="22" max="111" width="11.09765625" customWidth="1"/>
     <col min="112" max="1011" width="12.09765625" customWidth="1"/>
@@ -1039,7 +1041,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1049,10 +1051,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1064,29 +1066,29 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1098,20 +1100,20 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E01ACCD-5698-4424-95D5-93F796623CB6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="11.09765625" customWidth="1"/>
     <col min="3" max="3" width="10.796875" customWidth="1"/>
-    <col min="4" max="5" width="8.796875" style="2"/>
+    <col min="4" max="5" width="8.796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.09765625" customWidth="1"/>
     <col min="7" max="7" width="9.3984375" customWidth="1"/>
     <col min="8" max="8" width="9.8984375" customWidth="1"/>
-    <col min="9" max="9" width="9.09765625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="9.09765625" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.3984375" customWidth="1"/>
-    <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="17.796875" style="3" customWidth="1"/>
     <col min="13" max="21" width="10.09765625" customWidth="1"/>
     <col min="22" max="111" width="11.09765625" customWidth="1"/>
     <col min="112" max="1011" width="12.09765625" customWidth="1"/>
@@ -1119,7 +1121,7 @@
     <col min="10012" max="16384" width="14.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1129,10 +1131,10 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1144,29 +1146,29 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1178,31 +1180,31 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073C8F8E-56D4-4759-9B53-87C4A14D7ED7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="10.59765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.59765625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9.796875" style="3" customWidth="1"/>
     <col min="4" max="4" width="10.69921875" style="5" customWidth="1"/>
     <col min="5" max="5" width="9.8984375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G1" t="s">
         <v>28</v>

</xml_diff>